<commit_message>
README file update with the installation instructions
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29650A1-7408-462A-B302-A8F770F3F7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6848552A-E020-4910-BF86-D37FED3F0752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work Log" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="192">
   <si>
     <t>Date</t>
   </si>
@@ -529,6 +529,135 @@
   <si>
     <t>"Bridging the layers"</t>
   </si>
+  <si>
+    <t>Database Schema Optimization</t>
+  </si>
+  <si>
+    <t>Refined MySQL tables to ensure data integrity for incident severity mapping.</t>
+  </si>
+  <si>
+    <t>API Endpoint Development</t>
+  </si>
+  <si>
+    <t>Created Node.js routes to fetch total incident counts and hospitalization data.</t>
+  </si>
+  <si>
+    <t>Frontend Dashboard Integration</t>
+  </si>
+  <si>
+    <t>Integrated Recharts library into React to display the Incident Velocity Trend.</t>
+  </si>
+  <si>
+    <t>Component Styling</t>
+  </si>
+  <si>
+    <t>Designed the "SafeSight Intelligence Analytics" header and high-level stat cards.</t>
+  </si>
+  <si>
+    <t>Data Mapping: Fairmont Waterfront</t>
+  </si>
+  <si>
+    <t>Successfully mapped 391 historical records to the dashboard visualization layer.</t>
+  </si>
+  <si>
+    <t>Severity Distribution Logic</t>
+  </si>
+  <si>
+    <t>Programmed the pie chart logic to categorize "Critical" (83) and "High" (297) risks.</t>
+  </si>
+  <si>
+    <t>Departmental Risk Profiling</t>
+  </si>
+  <si>
+    <t>Developed the bar chart component to identify Housekeeping as the top risk area.</t>
+  </si>
+  <si>
+    <t>Research Access Configuration</t>
+  </si>
+  <si>
+    <t>Implemented "HR" research access level labels and restricted views in the UI.</t>
+  </si>
+  <si>
+    <t>Midterm Presentation Planning</t>
+  </si>
+  <si>
+    <t>Outlined the 10-minute presentation script for the full-stack system.</t>
+  </si>
+  <si>
+    <t>Navigation &amp; UI Logic</t>
+  </si>
+  <si>
+    <t>Finalized the top navigation bar links for Dashboard, Analytics, and WorkSafeBC.</t>
+  </si>
+  <si>
+    <t>Analytics Calculations</t>
+  </si>
+  <si>
+    <t>Verified the 97.1% risk probability metric against the 380 identified critical risks.</t>
+  </si>
+  <si>
+    <t>Script Refinement</t>
+  </si>
+  <si>
+    <t>Developed detailed speaking notes for role-based features and technical architecture.</t>
+  </si>
+  <si>
+    <t>Roadmap &amp; Worklog Finalization</t>
+  </si>
+  <si>
+    <t>Documented future AI implementation plans and finalized the Phase 2 development log.</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Technical Troubleshooting</t>
+  </si>
+  <si>
+    <t>Resolved backend connectivity issues and port 5000 configuration.</t>
+  </si>
+  <si>
+    <t>Full-Stack Integration</t>
+  </si>
+  <si>
+    <t>Successfully linked MySQL queries to React frontend components.</t>
+  </si>
+  <si>
+    <t>Data Visualization</t>
+  </si>
+  <si>
+    <t>Developed logic for Severity Distribution and Velocity Trend charts.</t>
+  </si>
+  <si>
+    <t>UX Design Analysis</t>
+  </si>
+  <si>
+    <t>Applied information hierarchy to prioritize Critical Risks (380) and Hospitalization (345) stats.</t>
+  </si>
+  <si>
+    <t>Business Logic</t>
+  </si>
+  <si>
+    <t>Identified Housekeeping as the primary risk area with 82+ incidents.</t>
+  </si>
+  <si>
+    <t>Content Creation</t>
+  </si>
+  <si>
+    <t>Structured a professional narrative for the solo midterm presentation.</t>
+  </si>
+  <si>
+    <t>"Dashboard stats and Recharts"</t>
+  </si>
+  <si>
+    <t>"AIDA framework for Dashboard"</t>
+  </si>
+  <si>
+    <t>"Departmental Risk Profile"</t>
+  </si>
+  <si>
+    <t>"10-minute presentation script"</t>
+  </si>
 </sst>
 </file>
 
@@ -537,7 +666,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -557,6 +686,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -607,7 +743,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -642,6 +778,12 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1362,103 +1504,233 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4">
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="3:4">
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="3:4">
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="3:4">
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="3:4">
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="3:4">
+    <row r="24" spans="1:4" ht="28.8">
+      <c r="A24" s="12">
+        <v>46063</v>
+      </c>
+      <c r="B24" s="14">
+        <v>2</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="28.8">
+      <c r="A25" s="12">
+        <v>46064</v>
+      </c>
+      <c r="B25" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28.8">
+      <c r="A26" s="12">
+        <v>46065</v>
+      </c>
+      <c r="B26" s="14">
+        <v>2</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="43.2">
+      <c r="A27" s="12">
+        <v>46066</v>
+      </c>
+      <c r="B27" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="43.2">
+      <c r="A28" s="12">
+        <v>46067</v>
+      </c>
+      <c r="B28" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="43.2">
+      <c r="A29" s="12">
+        <v>46068</v>
+      </c>
+      <c r="B29" s="14">
+        <v>2</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="43.2">
+      <c r="A30" s="12">
+        <v>46069</v>
+      </c>
+      <c r="B30" s="14">
+        <v>2</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="28.8">
+      <c r="A31" s="12">
+        <v>46070</v>
+      </c>
+      <c r="B31" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.8">
+      <c r="A32" s="12">
+        <v>46071</v>
+      </c>
+      <c r="B32" s="14">
+        <v>2</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="28.8">
+      <c r="A33" s="12">
+        <v>46072</v>
+      </c>
+      <c r="B33" s="14">
+        <v>1</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="28.8">
+      <c r="A34" s="12">
+        <v>46073</v>
+      </c>
+      <c r="B34" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="43.2">
+      <c r="A35" s="12">
+        <v>46074</v>
+      </c>
+      <c r="B35" s="14">
+        <v>2</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="43.2">
+      <c r="A36" s="12">
+        <v>46075</v>
+      </c>
+      <c r="B36" s="14">
+        <v>2</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
     </row>
-    <row r="38" spans="3:4">
+    <row r="38" spans="1:4">
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
     </row>
-    <row r="39" spans="3:4">
+    <row r="39" spans="1:4">
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
     </row>
-    <row r="40" spans="3:4">
+    <row r="40" spans="1:4">
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
     </row>
-    <row r="41" spans="3:4">
+    <row r="41" spans="1:4">
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="3:4">
+    <row r="42" spans="1:4">
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
     </row>
-    <row r="43" spans="3:4">
+    <row r="43" spans="1:4">
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="3:4">
+    <row r="44" spans="1:4">
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="3:4">
+    <row r="45" spans="1:4">
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="3:4">
+    <row r="46" spans="1:4">
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="3:4">
+    <row r="47" spans="1:4">
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="3:4">
+    <row r="48" spans="1:4">
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
     </row>
@@ -1800,7 +2072,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40EA87B-8D49-4A90-9FD7-CCB75014BEFC}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="8" customWidth="1"/>
@@ -2317,20 +2589,106 @@
         <v>96</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" ht="28.8">
       <c r="A31" s="8" t="s">
         <v>146</v>
       </c>
+      <c r="B31" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>176</v>
+      </c>
       <c r="D31" s="4" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="E31" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="28.8">
       <c r="A32" s="8" t="s">
         <v>146</v>
       </c>
+      <c r="B32" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>178</v>
+      </c>
       <c r="D32" s="4" t="s">
         <v>148</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="28.8">
+      <c r="A33" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="43.2">
+      <c r="A34" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28.8">
+      <c r="A35" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="28.8">
+      <c r="A36" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Documentation: Added Progress Report 2
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0F8750-848D-41D0-B4D5-9B200A091256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E915B735-7008-4591-B72E-F820412E2F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <sheet name="Prompts" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="223">
   <si>
     <t>Date</t>
   </si>
@@ -658,6 +657,99 @@
   </si>
   <si>
     <t>"10-minute presentation script"</t>
+  </si>
+  <si>
+    <t>Midterm Check-in</t>
+  </si>
+  <si>
+    <t>Advised to add a chatbot and a export version of worksafebc</t>
+  </si>
+  <si>
+    <t>Progress Report 2 Preparation</t>
+  </si>
+  <si>
+    <t>AI Service Setup</t>
+  </si>
+  <si>
+    <t>ML Model Training</t>
+  </si>
+  <si>
+    <t>Developed the Random Forest Classifier script using Scikit-Learn; implemented LabelEncoder to process categorical hotel data.</t>
+  </si>
+  <si>
+    <t>Initialized the AI_Service directory, configured a Python Virtual Environment (venv) to isolate Machine Learning dependencies.</t>
+  </si>
+  <si>
+    <t>Flask API Development</t>
+  </si>
+  <si>
+    <t>Created a Flask web server to host the ML model; established the /ai/predict-risk endpoint for real-time inference.</t>
+  </si>
+  <si>
+    <t>Backend Integration</t>
+  </si>
+  <si>
+    <t>Modified the Node.js server.js to act as an API Gateway; integrated Axios to fetch data from the Python service (Port 5001).</t>
+  </si>
+  <si>
+    <t>CORS &amp; Networking</t>
+  </si>
+  <si>
+    <t>Resolved Cross-Origin Resource Sharing (CORS) conflicts between the three running services (Ports 3000, 5000, and 5001).</t>
+  </si>
+  <si>
+    <t>Frontend UI Dev</t>
+  </si>
+  <si>
+    <t>Developed the Prediction.js React component; mapped AI "Risk Probabilities" to a visual dashboard for HR personnel.</t>
+  </si>
+  <si>
+    <t>3 Flash / Free Tier</t>
+  </si>
+  <si>
+    <t>Multi-service Integration</t>
+  </si>
+  <si>
+    <t>"How do I connect a Python Flask ML service to a Node.js Express backend?"</t>
+  </si>
+  <si>
+    <t>GPT-4o (Free)</t>
+  </si>
+  <si>
+    <t>Initial Code Logic</t>
+  </si>
+  <si>
+    <t>"Write a basic Random Forest Classifier for workplace safety incidents."</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>3.5 Sonnet (Free)</t>
+  </si>
+  <si>
+    <t>Technical Documentation</t>
+  </si>
+  <si>
+    <t>"Summarize my recent technical tasks into professional report language."</t>
+  </si>
+  <si>
+    <t>Troubleshooting</t>
+  </si>
+  <si>
+    <t>"Resolve CORS error between React and Flask using the flask-cors library."</t>
+  </si>
+  <si>
+    <t>Architectural Design: Defined the three-port strategy (3000, 5000, 5001) and integrated the bridge logic.</t>
+  </si>
+  <si>
+    <t>Algorithm Selection: Evaluated the generated script against hotel-specific data requirements to ensure model accuracy.</t>
+  </si>
+  <si>
+    <t>Communication: Refined the raw technical notes into the professional "Summary of Work" and "Technical Details" used in this report.</t>
+  </si>
+  <si>
+    <t>System Orchestration: Manually configured middleware in both services and verified the secure handshake across the local network.</t>
   </si>
 </sst>
 </file>
@@ -744,7 +836,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -785,6 +877,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -873,8 +983,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048574" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E1048574" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048573" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E1048573" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{7720FBCA-9D18-4AA6-AD20-22B601758C3E}" name="AI Tool Name" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{8D78E618-FCAF-4D63-B328-64EF4380AEB4}" name="Version / Account Type" dataDxfId="5"/>
@@ -1512,7 +1622,7 @@
       <c r="B24" s="14">
         <v>2</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="20" t="s">
         <v>149</v>
       </c>
       <c r="D24" s="13" t="s">
@@ -1526,7 +1636,7 @@
       <c r="B25" s="14">
         <v>1.5</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="20" t="s">
         <v>151</v>
       </c>
       <c r="D25" s="13" t="s">
@@ -1540,7 +1650,7 @@
       <c r="B26" s="14">
         <v>2</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="20" t="s">
         <v>153</v>
       </c>
       <c r="D26" s="13" t="s">
@@ -1554,7 +1664,7 @@
       <c r="B27" s="14">
         <v>1.5</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="20" t="s">
         <v>155</v>
       </c>
       <c r="D27" s="13" t="s">
@@ -1568,7 +1678,7 @@
       <c r="B28" s="14">
         <v>2.5</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="20" t="s">
         <v>157</v>
       </c>
       <c r="D28" s="13" t="s">
@@ -1582,24 +1692,24 @@
       <c r="B29" s="14">
         <v>2</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="20" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="43.2">
+    <row r="30" spans="1:4" ht="28.8">
       <c r="A30" s="12">
         <v>46069</v>
       </c>
       <c r="B30" s="14">
         <v>2</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="20" t="s">
         <v>162</v>
       </c>
     </row>
@@ -1610,10 +1720,10 @@
       <c r="B31" s="14">
         <v>1.5</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="20" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1624,10 +1734,10 @@
       <c r="B32" s="14">
         <v>2</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="20" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1638,10 +1748,10 @@
       <c r="B33" s="14">
         <v>1</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="20" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1652,10 +1762,10 @@
       <c r="B34" s="14">
         <v>2.5</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="20" t="s">
         <v>170</v>
       </c>
     </row>
@@ -1666,10 +1776,10 @@
       <c r="B35" s="14">
         <v>2</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="20" t="s">
         <v>172</v>
       </c>
     </row>
@@ -1680,43 +1790,121 @@
       <c r="B36" s="14">
         <v>2</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="20" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
+    <row r="37" spans="1:4" ht="57.6">
+      <c r="A37" s="12">
+        <v>46076</v>
+      </c>
+      <c r="B37" s="6">
+        <v>2</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="57.6">
+      <c r="A38" s="12">
+        <v>46077</v>
+      </c>
+      <c r="B38" s="6">
+        <v>1</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="43.2">
+      <c r="A39" s="12">
+        <v>46078</v>
+      </c>
+      <c r="B39" s="6">
+        <v>1</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="43.2">
+      <c r="A40" s="12">
+        <v>46079</v>
+      </c>
+      <c r="B40" s="6">
+        <v>1</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="28.8">
+      <c r="A41" s="12">
+        <v>46080</v>
+      </c>
+      <c r="B41" s="6">
+        <v>3</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="57.6">
+      <c r="A42" s="12">
+        <v>46081</v>
+      </c>
+      <c r="B42" s="6">
+        <v>1</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="57.6">
+      <c r="A43" s="12">
+        <v>46082</v>
+      </c>
+      <c r="B43" s="6">
+        <v>2</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="44" spans="1:4">
-      <c r="C44" s="2"/>
+      <c r="A44" s="12">
+        <v>46083</v>
+      </c>
+      <c r="B44" s="6">
+        <v>2</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>194</v>
+      </c>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4">
@@ -2073,7 +2261,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40EA87B-8D49-4A90-9FD7-CCB75014BEFC}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="8" customWidth="1"/>
@@ -2690,6 +2878,74 @@
       </c>
       <c r="E36" s="4" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="57.6">
+      <c r="A37" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="57.6">
+      <c r="A38" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="57.6">
+      <c r="A39" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="57.6">
+      <c r="A40" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: finalize Progress Report 3 and update AI usage documentation
Refined project methodology to focus on EIIR (Form 52E40) automation and updated the Work Log for Phase 4 milestones.
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E915B735-7008-4591-B72E-F820412E2F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6619612C-8D63-4958-93BD-CB6108E6DE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="234">
   <si>
     <t>Date</t>
   </si>
@@ -751,6 +751,81 @@
   <si>
     <t>System Orchestration: Manually configured middleware in both services and verified the secure handshake across the local network.</t>
   </si>
+  <si>
+    <t>Progress Report 3 Preparation</t>
+  </si>
+  <si>
+    <t>Refining Random Forest Model and Shift/Department hotspot mapping.</t>
+  </si>
+  <si>
+    <t>AI Service testing completed.</t>
+  </si>
+  <si>
+    <t>Researching WorkSafeBC EIIR (Form 52E40) PDF structure and XFA requirements.</t>
+  </si>
+  <si>
+    <t>Decided to pivot from Form 7.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Implementing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>pdf-lib</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in the backend and creating XFA field mapping logic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Established </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>reportController.js</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Developing Frontend "Export" component and handling binary BLOB data streams.</t>
+  </si>
+  <si>
+    <t>PDF download button implemented.</t>
+  </si>
+  <si>
+    <t>Troubleshooting API Handshake and resolving "Database Error" in report generation.</t>
+  </si>
+  <si>
+    <t>In Progress: Debugging 500 error shown in logs.</t>
+  </si>
 </sst>
 </file>
 
@@ -759,7 +834,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -783,6 +858,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -836,7 +918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -878,23 +960,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -970,8 +1040,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}" name="Table1" displayName="Table1" ref="A1:D130" totalsRowShown="0">
-  <autoFilter ref="A1:D130" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}" name="Table1" displayName="Table1" ref="A1:D126" totalsRowShown="0">
+  <autoFilter ref="A1:D126" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{5ABDF1AC-6CA2-4D3D-BED1-ABBE8632EF5A}" name="Date" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{48C587D8-0357-4367-9662-FE4DF7A0731E}" name="Number of Hours" dataDxfId="11"/>
@@ -1307,7 +1377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24.5546875" style="1" customWidth="1"/>
@@ -1622,7 +1692,7 @@
       <c r="B24" s="14">
         <v>2</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="15" t="s">
         <v>149</v>
       </c>
       <c r="D24" s="13" t="s">
@@ -1636,7 +1706,7 @@
       <c r="B25" s="14">
         <v>1.5</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="15" t="s">
         <v>151</v>
       </c>
       <c r="D25" s="13" t="s">
@@ -1650,7 +1720,7 @@
       <c r="B26" s="14">
         <v>2</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="15" t="s">
         <v>153</v>
       </c>
       <c r="D26" s="13" t="s">
@@ -1664,7 +1734,7 @@
       <c r="B27" s="14">
         <v>1.5</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="15" t="s">
         <v>155</v>
       </c>
       <c r="D27" s="13" t="s">
@@ -1678,7 +1748,7 @@
       <c r="B28" s="14">
         <v>2.5</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="15" t="s">
         <v>157</v>
       </c>
       <c r="D28" s="13" t="s">
@@ -1692,10 +1762,10 @@
       <c r="B29" s="14">
         <v>2</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="15" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1706,10 +1776,10 @@
       <c r="B30" s="14">
         <v>2</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="15" t="s">
         <v>162</v>
       </c>
     </row>
@@ -1720,10 +1790,10 @@
       <c r="B31" s="14">
         <v>1.5</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="15" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1734,10 +1804,10 @@
       <c r="B32" s="14">
         <v>2</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C32" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="15" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1748,10 +1818,10 @@
       <c r="B33" s="14">
         <v>1</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="15" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1762,24 +1832,24 @@
       <c r="B34" s="14">
         <v>2.5</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="15" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="43.2">
+    <row r="35" spans="1:4" ht="28.8">
       <c r="A35" s="12">
         <v>46074</v>
       </c>
       <c r="B35" s="14">
         <v>2</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="15" t="s">
         <v>172</v>
       </c>
     </row>
@@ -1790,10 +1860,10 @@
       <c r="B36" s="14">
         <v>2</v>
       </c>
-      <c r="C36" s="20" t="s">
+      <c r="C36" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="D36" s="15" t="s">
         <v>174</v>
       </c>
     </row>
@@ -1804,10 +1874,10 @@
       <c r="B37" s="6">
         <v>2</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="D37" s="2" t="s">
         <v>198</v>
       </c>
     </row>
@@ -1818,10 +1888,10 @@
       <c r="B38" s="6">
         <v>1</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D38" s="2" t="s">
         <v>197</v>
       </c>
     </row>
@@ -1832,10 +1902,10 @@
       <c r="B39" s="6">
         <v>1</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="C39" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="D39" s="2" t="s">
         <v>200</v>
       </c>
     </row>
@@ -1846,10 +1916,10 @@
       <c r="B40" s="6">
         <v>1</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="2" t="s">
         <v>202</v>
       </c>
     </row>
@@ -1860,38 +1930,38 @@
       <c r="B41" s="6">
         <v>3</v>
       </c>
-      <c r="C41" s="19" t="s">
+      <c r="C41" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="D41" s="15" t="s">
+      <c r="D41" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="57.6">
+    <row r="42" spans="1:4" ht="43.2">
       <c r="A42" s="12">
         <v>46081</v>
       </c>
       <c r="B42" s="6">
         <v>1</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="C42" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="57.6">
+    <row r="43" spans="1:4" ht="43.2">
       <c r="A43" s="12">
         <v>46082</v>
       </c>
       <c r="B43" s="6">
         <v>2</v>
       </c>
-      <c r="C43" s="18" t="s">
+      <c r="C43" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D43" s="15" t="s">
+      <c r="D43" s="2" t="s">
         <v>206</v>
       </c>
     </row>
@@ -1907,83 +1977,141 @@
       </c>
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="1:4">
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-    </row>
-    <row r="48" spans="1:4">
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-    </row>
-    <row r="49" spans="3:4">
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="3:4">
-      <c r="C50" s="2"/>
+    <row r="45" spans="1:4" ht="28.8">
+      <c r="A45" s="12">
+        <v>46084</v>
+      </c>
+      <c r="B45" s="6">
+        <v>3</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="31.2" customHeight="1">
+      <c r="A46" s="12">
+        <v>46085</v>
+      </c>
+      <c r="B46" s="6">
+        <v>2</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D46" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="28.8">
+      <c r="A47" s="12">
+        <v>46086</v>
+      </c>
+      <c r="B47" s="6">
+        <v>2</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D47" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="28.2" customHeight="1">
+      <c r="A48" s="12">
+        <v>46087</v>
+      </c>
+      <c r="B48" s="6">
+        <v>2</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D48" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="43.2">
+      <c r="A49" s="12">
+        <v>46089</v>
+      </c>
+      <c r="B49" s="6">
+        <v>2</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="12">
+        <v>46090</v>
+      </c>
+      <c r="B50" s="6">
+        <v>2</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>223</v>
+      </c>
       <c r="D50" s="2"/>
     </row>
-    <row r="51" spans="3:4">
+    <row r="51" spans="1:4">
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
     </row>
-    <row r="52" spans="3:4">
+    <row r="52" spans="1:4">
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
     </row>
-    <row r="53" spans="3:4">
+    <row r="53" spans="1:4">
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="3:4">
+    <row r="54" spans="1:4">
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="3:4">
+    <row r="55" spans="1:4">
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="3:4">
+    <row r="56" spans="1:4">
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
     </row>
-    <row r="57" spans="3:4">
+    <row r="57" spans="1:4">
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
     </row>
-    <row r="58" spans="3:4">
+    <row r="58" spans="1:4">
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
     </row>
-    <row r="59" spans="3:4">
+    <row r="59" spans="1:4">
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
     </row>
-    <row r="60" spans="3:4">
+    <row r="60" spans="1:4">
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
     </row>
-    <row r="61" spans="3:4">
+    <row r="61" spans="1:4">
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
     </row>
-    <row r="62" spans="3:4">
+    <row r="62" spans="1:4">
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
     </row>
-    <row r="63" spans="3:4">
+    <row r="63" spans="1:4">
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
     </row>
-    <row r="64" spans="3:4">
+    <row r="64" spans="1:4">
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
     </row>
@@ -2234,22 +2362,6 @@
     <row r="126" spans="3:4">
       <c r="C126" s="2"/>
       <c r="D126" s="2"/>
-    </row>
-    <row r="127" spans="3:4">
-      <c r="C127" s="2"/>
-      <c r="D127" s="2"/>
-    </row>
-    <row r="128" spans="3:4">
-      <c r="C128" s="2"/>
-      <c r="D128" s="2"/>
-    </row>
-    <row r="129" spans="3:4">
-      <c r="C129" s="2"/>
-      <c r="D129" s="2"/>
-    </row>
-    <row r="130" spans="3:4">
-      <c r="C130" s="2"/>
-      <c r="D130" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2881,70 +2993,70 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="57.6">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="15" t="s">
         <v>208</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="E37" s="17" t="s">
+      <c r="E37" s="16" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="57.6">
-      <c r="A38" s="16" t="s">
+      <c r="A38" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="16" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="57.6">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="C39" s="16" t="s">
+      <c r="C39" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="E39" s="17" t="s">
+      <c r="E39" s="16" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="57.6">
-      <c r="A40" s="16" t="s">
+      <c r="A40" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E40" s="16" t="s">
         <v>222</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update AI usage documentation
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6619612C-8D63-4958-93BD-CB6108E6DE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC75D8C-63B3-44E1-BA9F-AD2ED1DF7E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work Log" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="265">
   <si>
     <t>Date</t>
   </si>
@@ -826,6 +826,126 @@
   <si>
     <t>In Progress: Debugging 500 error shown in logs.</t>
   </si>
+  <si>
+    <t>Code Analysis &amp; Documentation</t>
+  </si>
+  <si>
+    <t>"How do I programmatically fill a WorkSafeBC EIIR PDF form using JavaScript?"</t>
+  </si>
+  <si>
+    <t>Debugging / Log Interpretation</t>
+  </si>
+  <si>
+    <t>"Why does pdf-lib return 'Invalid Object Reference' when loading an encrypted government PDF?"</t>
+  </si>
+  <si>
+    <t>Architecture Design</t>
+  </si>
+  <si>
+    <t>"How to download a PDF from a Node.js backend to a React frontend without saving it to disk?"</t>
+  </si>
+  <si>
+    <t>Troubleshooting corrupted PDF downloads and binary data handling.</t>
+  </si>
+  <si>
+    <t>Code Refactoring</t>
+  </si>
+  <si>
+    <t>"Update my Express.js SQL query to use 'incident_id' instead of 'id' and sync with the frontend."</t>
+  </si>
+  <si>
+    <t>Systematic Debugging</t>
+  </si>
+  <si>
+    <t>"My GET request to /api/reports/generate/13 is returning a 404. Check my server.js route order."</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Prevented hours of wasted effort by identifying early that standard </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>getFields()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> methods would fail, requiring a "Deep Mapping" approach.</t>
+    </r>
+  </si>
+  <si>
+    <t>Engineered a "Zero-Storage" flow, ensuring sensitive data exists only in temporary memory, enhancing user data privacy.</t>
+  </si>
+  <si>
+    <t>Guaranteed 100% accuracy in data-to-field mapping, ensuring the correct incident record is always injected into the legal export.</t>
+  </si>
+  <si>
+    <t>Provided a systematic framework to isolate failures between the Express router and the MySQL connection pool.</t>
+  </si>
+  <si>
+    <t>GPT-5.3 / Free Plan</t>
+  </si>
+  <si>
+    <t>Concept clarification and debugging guidance</t>
+  </si>
+  <si>
+    <t>"Prompts describing API routing errors, PDF generation issues, and data flow between the React frontend, Node.js backend, and MySQL database"</t>
+  </si>
+  <si>
+    <t>Applied the conceptual guidance to troubleshoot system integration issues, tested solutions using developer tools and Postman, and implemented the final working logic in the application</t>
+  </si>
+  <si>
+    <t>GitHub Copilot</t>
+  </si>
+  <si>
+    <t>Student / IDE Integration</t>
+  </si>
+  <si>
+    <t>Code suggestion and auto-completion</t>
+  </si>
+  <si>
+    <t>Reviewed, modified, and optimized suggested code to ensure compatibility with the microservices architecture and database schema</t>
+  </si>
+  <si>
+    <t>Python NLP Libraries (via AI assistance)</t>
+  </si>
+  <si>
+    <t>Local Development Environment</t>
+  </si>
+  <si>
+    <t>Natural Language Processing preparation</t>
+  </si>
+  <si>
+    <t>Designed how the NLP layer integrates with the incident reporting pipeline and adapted outputs to match regulatory documentation standards</t>
+  </si>
+  <si>
+    <t>Technical writing and documentation refinement</t>
+  </si>
+  <si>
+    <t>"Context-based code suggestions for JavaScript, Express.js routing, and React component logic"</t>
+  </si>
+  <si>
+    <t>"Prompts related to sanitizing and improving incident narrative descriptions for professional reporting"</t>
+  </si>
+  <si>
+    <t>"Prompts requesting restructuring of technical descriptions, summaries, and professional wording for project documentation and reports"</t>
+  </si>
 </sst>
 </file>
 
@@ -834,7 +954,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -865,6 +985,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -918,7 +1044,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -965,6 +1091,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2373,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40EA87B-8D49-4A90-9FD7-CCB75014BEFC}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="8" customWidth="1"/>
@@ -3060,7 +3192,161 @@
         <v>222</v>
       </c>
     </row>
+    <row r="41" spans="1:5" ht="57.6">
+      <c r="A41" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E41" s="17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="57.6">
+      <c r="A42" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="57.6">
+      <c r="A43" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="57.6">
+      <c r="A44" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="57.6">
+      <c r="A45" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="86.4">
+      <c r="A46" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="57.6">
+      <c r="A47" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="72">
+      <c r="A48" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="86.4">
+      <c r="A49" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Progress Report 4 submission
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC75D8C-63B3-44E1-BA9F-AD2ED1DF7E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF875E0-C971-4333-A96B-16F5A2643760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="305">
   <si>
     <t>Date</t>
   </si>
@@ -946,6 +946,366 @@
   <si>
     <t>"Prompts requesting restructuring of technical descriptions, summaries, and professional wording for project documentation and reports"</t>
   </si>
+  <si>
+    <t>Progress Report 5 Preparation</t>
+  </si>
+  <si>
+    <t>Regulatory Form Pivot &amp; Logic Mapping</t>
+  </si>
+  <si>
+    <t>PDF Document Engineering</t>
+  </si>
+  <si>
+    <t>Excel Analytics Implementation</t>
+  </si>
+  <si>
+    <t>Backend Infrastructure Refactor</t>
+  </si>
+  <si>
+    <t>UI Integration &amp; Final Testing</t>
+  </si>
+  <si>
+    <t>Added dual-action export buttons to the React Frontend. Verified binary blob handling and performed full-stack verification of the reporting suite.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Successfully redirected the project to automate the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>WorkSafeBC EIIR (Form 52E40). Mapped SQL fields to the specific regulatory layout.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Integrated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>pdfkit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and implemented coordinate-based rendering to ensure document structural integrity and Fairmont branding.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Developed the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>exceljs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> export route. Programmed data transformation logic to convert database values into human-readable analytics.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Migrated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>mysql2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> connection pool to Promise-based architecture. Optimized dashboard query performance to fix data sync issues.</t>
+    </r>
+  </si>
+  <si>
+    <t>Gemini (Google)</t>
+  </si>
+  <si>
+    <t>Multi-turn Code Generation &amp; Troubleshooting</t>
+  </si>
+  <si>
+    <t>Technical documentation, debugging explanations, and system design clarification</t>
+  </si>
+  <si>
+    <t>Context-aware code completion and inline suggestions</t>
+  </si>
+  <si>
+    <t>Perplexity AI</t>
+  </si>
+  <si>
+    <t>Free Plan</t>
+  </si>
+  <si>
+    <t>AI-assisted research and technical reference lookup</t>
+  </si>
+  <si>
+    <t>Claude (Anthropic)</t>
+  </si>
+  <si>
+    <t>Free / Web Access</t>
+  </si>
+  <si>
+    <t>Structured reasoning and code explanation</t>
+  </si>
+  <si>
+    <t>Google Colab / Python NLP Tools</t>
+  </si>
+  <si>
+    <t>Free Tier</t>
+  </si>
+  <si>
+    <t>Natural Language Processing experimentation</t>
+  </si>
+  <si>
+    <t>Postman AI Assistance</t>
+  </si>
+  <si>
+    <t>API testing and request validation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">“Develop an Excel export route using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>exceljs for analytics; refactor Node.js backend to async/await to resolve dashboard sync issues; and map SQL data to a custom PDF layout mirroring WorkSafeBC Form 52E40.”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Directed the strategic pivot from generic reporting to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>automated regulatory compliance (Form 52E40). Identified and resolved the architectural conflict between legacy callbacks and modern promises, restoring dashboard functionality. Designed the dual-stream UI logic to support both regulatory reporting and internal analytics.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Prompts requesting refinement of system architecture explanations, troubleshooting </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>API routing, PDF generation logic, and frontend–backend data synchronization.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Interpreted and validated AI outputs against the implemented system. Adapted explanations to align with the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Node.js–React–MySQL microservices architecture and ensured documentation accurately reflected the developed solution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Auto-suggestions for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Express.js routes, React component state management, and JavaScript data transformation logic while writing backend and frontend code.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reviewed and refactored generated snippets to meet project architecture requirements. Ensured compatibility with the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>database schema, API routes, and compliance reporting workflow.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Queries regarding </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>XFA PDF form structures, government form automation approaches, and handling binary streams (Blob responses) in web applications.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Validated technical approaches and translated research findings into practical implementation strategies within the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PDF generation and export pipeline.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Prompts requesting explanations of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>asynchronous JavaScript patterns, Promise-based database handling, and structured debugging strategies.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Applied reasoning outputs to restructure backend logic, improving </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>database query performance and error handling across API routes.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Prompts exploring </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>text sanitization and professional rewriting of incident descriptions before inserting them into compliance reports.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Designed the concept of an </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI-powered narrative refinement layer to convert raw incident descriptions into professional language suitable for regulatory documentation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Prompts and automated suggestions for debugging </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>REST API endpoints, request headers, and route mismatches during integration testing.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Used insights from testing to identify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>API handshake and routing issues, ensuring correct communication between frontend requests and backend services.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -954,7 +1314,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -991,6 +1351,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1044,7 +1411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1092,11 +1459,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1108,6 +1478,18 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1146,18 +1528,6 @@
       </font>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
@@ -1175,24 +1545,24 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}" name="Table1" displayName="Table1" ref="A1:D126" totalsRowShown="0">
   <autoFilter ref="A1:D126" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5ABDF1AC-6CA2-4D3D-BED1-ABBE8632EF5A}" name="Date" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{48C587D8-0357-4367-9662-FE4DF7A0731E}" name="Number of Hours" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{423E5E18-754F-4F31-A0AF-8A6961646D3E}" name="Description" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{4D463411-D60A-45E9-A354-72F630B4F08F}" name="Remarks" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{5ABDF1AC-6CA2-4D3D-BED1-ABBE8632EF5A}" name="Date" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{48C587D8-0357-4367-9662-FE4DF7A0731E}" name="Number of Hours" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{423E5E18-754F-4F31-A0AF-8A6961646D3E}" name="Description" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{4D463411-D60A-45E9-A354-72F630B4F08F}" name="Remarks" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048573" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E1048573" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048572" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:E1048572" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7720FBCA-9D18-4AA6-AD20-22B601758C3E}" name="AI Tool Name" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{8D78E618-FCAF-4D63-B328-64EF4380AEB4}" name="Version / Account Type" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{B99F606B-3981-4DF0-80B0-82F9716EEB6E}" name="Specific Feature Used" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{C60CFB0A-096D-48E4-BBCB-28DF6594EBFA}" name="Prompt Used (Summary)" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{5423605D-7B52-4200-9789-A3D7EF34731D}" name="Value Addition (Student Contribution)" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{7720FBCA-9D18-4AA6-AD20-22B601758C3E}" name="AI Tool Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{8D78E618-FCAF-4D63-B328-64EF4380AEB4}" name="Version / Account Type" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{B99F606B-3981-4DF0-80B0-82F9716EEB6E}" name="Specific Feature Used" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{C60CFB0A-096D-48E4-BBCB-28DF6594EBFA}" name="Prompt Used (Summary)" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{5423605D-7B52-4200-9789-A3D7EF34731D}" name="Value Addition (Student Contribution)" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2191,28 +2561,86 @@
       </c>
       <c r="D50" s="2"/>
     </row>
-    <row r="51" spans="1:4">
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-    </row>
-    <row r="52" spans="1:4">
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-    </row>
-    <row r="53" spans="1:4">
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
+    <row r="51" spans="1:4" ht="57.6">
+      <c r="A51" s="12">
+        <v>46091</v>
+      </c>
+      <c r="B51" s="6">
+        <v>2</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="57.6">
+      <c r="A52" s="12">
+        <v>46092</v>
+      </c>
+      <c r="B52" s="6">
+        <v>2</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="D52" s="18" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="57.6">
+      <c r="A53" s="12">
+        <v>46093</v>
+      </c>
+      <c r="B53" s="6">
+        <v>3</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="D53" s="18" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="57.6">
+      <c r="A54" s="12">
+        <v>46094</v>
+      </c>
+      <c r="B54" s="6">
+        <v>2</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="D54" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="57.6">
+      <c r="A55" s="12">
+        <v>46095</v>
+      </c>
+      <c r="B55" s="6">
+        <v>2</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="D55" s="18" t="s">
+        <v>271</v>
+      </c>
     </row>
     <row r="56" spans="1:4">
-      <c r="C56" s="2"/>
+      <c r="A56" s="12">
+        <v>46096</v>
+      </c>
+      <c r="B56" s="6">
+        <v>3</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>265</v>
+      </c>
       <c r="D56" s="2"/>
     </row>
     <row r="57" spans="1:4">
@@ -2505,7 +2933,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40EA87B-8D49-4A90-9FD7-CCB75014BEFC}">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="8" customWidth="1"/>
@@ -3205,7 +3633,7 @@
       <c r="D41" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E41" s="17" t="s">
+      <c r="E41" s="4" t="s">
         <v>245</v>
       </c>
     </row>
@@ -3295,10 +3723,10 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="57.6">
-      <c r="A47" s="18" t="s">
+      <c r="A47" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="17" t="s">
         <v>254</v>
       </c>
       <c r="C47" s="3" t="s">
@@ -3312,7 +3740,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="72">
-      <c r="A48" s="18" t="s">
+      <c r="A48" s="17" t="s">
         <v>257</v>
       </c>
       <c r="B48" s="11" t="s">
@@ -3329,10 +3757,10 @@
       </c>
     </row>
     <row r="49" spans="1:5" ht="86.4">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="17" t="s">
         <v>249</v>
       </c>
       <c r="C49" s="3" t="s">
@@ -3343,6 +3771,125 @@
       </c>
       <c r="E49" s="2" t="s">
         <v>260</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="129.6">
+      <c r="A50" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="B50" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="115.2">
+      <c r="A51" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>278</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="115.2">
+      <c r="A52" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="100.8">
+      <c r="A53" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="B53" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>282</v>
+      </c>
+      <c r="D53" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="100.8">
+      <c r="A54" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="B54" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="86.4">
+      <c r="A55" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="86.4">
+      <c r="A56" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="B56" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="E56" s="19" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Progress Report 5: Integrated RandomForest ML Engine and implemented Dual-Mode Dashboard Architecture
</commit_message>
<xml_diff>
--- a/DocumentAndReports/Work Log.xlsx
+++ b/DocumentAndReports/Work Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandali Silva\Documents\GitHub\W26_4495_S2_SandaliS\DocumentAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF875E0-C971-4333-A96B-16F5A2643760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237F2F61-533B-40F2-88BC-0C44C2CBFCEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work Log" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="355">
   <si>
     <t>Date</t>
   </si>
@@ -1306,6 +1306,156 @@
       <t>API handshake and routing issues, ensuring correct communication between frontend requests and backend services.</t>
     </r>
   </si>
+  <si>
+    <t>Progress Report 4 Preparation</t>
+  </si>
+  <si>
+    <t>Developed and configured RandomForest Classifier using Python and Scikit-Learn for predictive risk analysis</t>
+  </si>
+  <si>
+    <t>Established core ML model for handling categorical safety data</t>
+  </si>
+  <si>
+    <t>Performed feature engineering using Label Encoding to convert categorical variables (departments, shifts, incidents) into numerical format</t>
+  </si>
+  <si>
+    <t>Improved model’s ability to detect hidden risk patterns</t>
+  </si>
+  <si>
+    <t>Implemented predict_proba() to simulate future 30-day risk scenarios and generate probability-based outputs</t>
+  </si>
+  <si>
+    <t>Enabled proactive forecasting instead of reactive analysis</t>
+  </si>
+  <si>
+    <t>Designed ML output metrics including Confidence Score (%) and Risk Levels (Stable, Elevated, High)</t>
+  </si>
+  <si>
+    <t>Enhanced interpretability of AI predictions for decision-making</t>
+  </si>
+  <si>
+    <t>Built and tested Flask API to integrate ML engine with React frontend (AI service on port 5001)</t>
+  </si>
+  <si>
+    <t>Achieved real-time communication between frontend and AI backend</t>
+  </si>
+  <si>
+    <t>Implemented and refined Split-View Dashboard using React state management and conditional rendering</t>
+  </si>
+  <si>
+    <t>Improved usability by separating operational and strategic views</t>
+  </si>
+  <si>
+    <t>Integrated ML predictions into Intelligence View with Recharts visualizations and optimized backend queries</t>
+  </si>
+  <si>
+    <t>Ensured seamless display of predictive insights with high performance</t>
+  </si>
+  <si>
+    <t>Technical explanation, code structuring, debugging assistance</t>
+  </si>
+  <si>
+    <t>Requested help to structure ML integration, refine backend logic, and format technical documentation</t>
+  </si>
+  <si>
+    <t>Interpreted outputs, customized logic to project needs, and ensured proper integration with SafeSight architecture</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Gemini 3 Flash / Free Tier</t>
+  </si>
+  <si>
+    <t>Multi-turn code generation &amp; system design suggestions</t>
+  </si>
+  <si>
+    <t>Generated ideas for AI integration, dashboard architecture, and backend optimization</t>
+  </si>
+  <si>
+    <t>Critically evaluated suggestions and adapted them into a working full-stack solution</t>
+  </si>
+  <si>
+    <t>Claude 3 / Free Tier</t>
+  </si>
+  <si>
+    <t>Long-form reasoning &amp; documentation refinement</t>
+  </si>
+  <si>
+    <t>Used to refine explanations of ML workflow, predictive analytics, and research writing clarity</t>
+  </si>
+  <si>
+    <t>Improved academic quality, ensured clarity, and aligned content with project objectives</t>
+  </si>
+  <si>
+    <t>Scikit-Learn (AI Library)</t>
+  </si>
+  <si>
+    <t>Latest Stable Version</t>
+  </si>
+  <si>
+    <t>RandomForest Classifier &amp; predict_proba()</t>
+  </si>
+  <si>
+    <t>Implemented ML model for classification and probability-based forecasting</t>
+  </si>
+  <si>
+    <t>Designed model logic, selected features, trained model, and validated outputs</t>
+  </si>
+  <si>
+    <t>Postman</t>
+  </si>
+  <si>
+    <t>Desktop App / Free</t>
+  </si>
+  <si>
+    <t>API testing &amp; endpoint validation</t>
+  </si>
+  <si>
+    <t>Tested Flask API endpoints for ML predictions and backend integration</t>
+  </si>
+  <si>
+    <t>Ensured reliable API communication and debugged request/response issues</t>
+  </si>
+  <si>
+    <t>Free / Student Access</t>
+  </si>
+  <si>
+    <t>Code auto-completion &amp; suggestions</t>
+  </si>
+  <si>
+    <t>Assisted in writing Python, React, and Node.js code snippets</t>
+  </si>
+  <si>
+    <t>Reviewed, modified, and validated generated code to ensure correctness</t>
+  </si>
+  <si>
+    <t>Recharts</t>
+  </si>
+  <si>
+    <t>Open Source Library</t>
+  </si>
+  <si>
+    <t>Data visualization (Radar, Stacked Bar charts)</t>
+  </si>
+  <si>
+    <t>Used for mapping ML outputs into visual analytics</t>
+  </si>
+  <si>
+    <t>Designed meaningful visual representations for predictive insights</t>
+  </si>
+  <si>
+    <t>Axios</t>
+  </si>
+  <si>
+    <t>API integration &amp; async data fetching</t>
+  </si>
+  <si>
+    <t>Used to fetch ML predictions from Flask backend into React frontend</t>
+  </si>
+  <si>
+    <t>Implemented efficient data flow and ensured real-time updates</t>
+  </si>
 </sst>
 </file>
 
@@ -1314,7 +1464,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1351,13 +1501,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1411,7 +1554,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1461,12 +1604,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1542,8 +1679,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}" name="Table1" displayName="Table1" ref="A1:D126" totalsRowShown="0">
-  <autoFilter ref="A1:D126" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}" name="Table1" displayName="Table1" ref="A1:D124" totalsRowShown="0">
+  <autoFilter ref="A1:D124" xr:uid="{41F59F99-6A6B-4C90-994D-BBFEB2BDE46C}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{5ABDF1AC-6CA2-4D3D-BED1-ABBE8632EF5A}" name="Date" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{48C587D8-0357-4367-9662-FE4DF7A0731E}" name="Number of Hours" dataDxfId="4"/>
@@ -1555,8 +1692,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048572" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:E1048572" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}" name="Table3" displayName="Table3" ref="A1:E1048571" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:E1048571" xr:uid="{62A78FFA-69C1-4830-8948-7A15783C8983}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{7720FBCA-9D18-4AA6-AD20-22B601758C3E}" name="AI Tool Name" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{8D78E618-FCAF-4D63-B328-64EF4380AEB4}" name="Version / Account Type" dataDxfId="9"/>
@@ -1879,7 +2016,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24.5546875" style="1" customWidth="1"/>
@@ -2568,10 +2705,10 @@
       <c r="B51" s="6">
         <v>2</v>
       </c>
-      <c r="C51" s="18" t="s">
+      <c r="C51" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="D51" s="18" t="s">
+      <c r="D51" s="2" t="s">
         <v>272</v>
       </c>
     </row>
@@ -2582,10 +2719,10 @@
       <c r="B52" s="6">
         <v>2</v>
       </c>
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="D52" s="18" t="s">
+      <c r="D52" s="2" t="s">
         <v>273</v>
       </c>
     </row>
@@ -2596,10 +2733,10 @@
       <c r="B53" s="6">
         <v>3</v>
       </c>
-      <c r="C53" s="18" t="s">
+      <c r="C53" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="D53" s="18" t="s">
+      <c r="D53" s="2" t="s">
         <v>274</v>
       </c>
     </row>
@@ -2610,10 +2747,10 @@
       <c r="B54" s="6">
         <v>2</v>
       </c>
-      <c r="C54" s="18" t="s">
+      <c r="C54" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D54" s="18" t="s">
+      <c r="D54" s="2" t="s">
         <v>275</v>
       </c>
     </row>
@@ -2624,10 +2761,10 @@
       <c r="B55" s="6">
         <v>2</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D55" s="18" t="s">
+      <c r="D55" s="2" t="s">
         <v>271</v>
       </c>
     </row>
@@ -2639,103 +2776,182 @@
         <v>3</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57" spans="1:4" ht="43.2">
+      <c r="A57" s="12">
+        <v>46097</v>
+      </c>
+      <c r="B57" s="11">
+        <v>4</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="57.6">
+      <c r="A58" s="12">
+        <v>46098</v>
+      </c>
+      <c r="B58" s="11">
+        <v>4</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="43.2">
+      <c r="A59" s="12">
+        <v>46099</v>
+      </c>
+      <c r="B59" s="11">
+        <v>3</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="43.2">
+      <c r="A60" s="12">
+        <v>46100</v>
+      </c>
+      <c r="B60" s="11">
+        <v>3</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="43.2">
+      <c r="A61" s="12">
+        <v>46101</v>
+      </c>
+      <c r="B61" s="11">
+        <v>2.5</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="43.2">
+      <c r="A62" s="12">
+        <v>46102</v>
+      </c>
+      <c r="B62" s="11">
+        <v>3</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="43.2">
+      <c r="A63" s="12">
+        <v>46103</v>
+      </c>
+      <c r="B63" s="11">
+        <v>3</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="12">
+        <v>46104</v>
+      </c>
+      <c r="B64" s="6">
+        <v>3</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D56" s="2"/>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-    </row>
-    <row r="58" spans="1:4">
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-    </row>
-    <row r="59" spans="1:4">
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="C64" s="2"/>
       <c r="D64" s="2"/>
     </row>
-    <row r="65" spans="3:4">
+    <row r="65" spans="1:4">
+      <c r="A65" s="12"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
     </row>
-    <row r="66" spans="3:4">
+    <row r="66" spans="1:4">
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
     </row>
-    <row r="67" spans="3:4">
+    <row r="67" spans="1:4">
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
     </row>
-    <row r="68" spans="3:4">
+    <row r="68" spans="1:4">
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
     </row>
-    <row r="69" spans="3:4">
+    <row r="69" spans="1:4">
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
     </row>
-    <row r="70" spans="3:4">
+    <row r="70" spans="1:4">
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
     </row>
-    <row r="71" spans="3:4">
+    <row r="71" spans="1:4">
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
     </row>
-    <row r="72" spans="3:4">
+    <row r="72" spans="1:4">
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
     </row>
-    <row r="73" spans="3:4">
+    <row r="73" spans="1:4">
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
     </row>
-    <row r="74" spans="3:4">
+    <row r="74" spans="1:4">
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
     </row>
-    <row r="75" spans="3:4">
+    <row r="75" spans="1:4">
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
     </row>
-    <row r="76" spans="3:4">
+    <row r="76" spans="1:4">
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
     </row>
-    <row r="77" spans="3:4">
+    <row r="77" spans="1:4">
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
     </row>
-    <row r="78" spans="3:4">
+    <row r="78" spans="1:4">
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
     </row>
-    <row r="79" spans="3:4">
+    <row r="79" spans="1:4">
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
     </row>
-    <row r="80" spans="3:4">
+    <row r="80" spans="1:4">
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
     </row>
@@ -2914,14 +3130,6 @@
     <row r="124" spans="3:4">
       <c r="C124" s="2"/>
       <c r="D124" s="2"/>
-    </row>
-    <row r="125" spans="3:4">
-      <c r="C125" s="2"/>
-      <c r="D125" s="2"/>
-    </row>
-    <row r="126" spans="3:4">
-      <c r="C126" s="2"/>
-      <c r="D126" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2933,7 +3141,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40EA87B-8D49-4A90-9FD7-CCB75014BEFC}">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="8" customWidth="1"/>
@@ -3774,122 +3982,258 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="129.6">
-      <c r="A50" s="19" t="s">
+      <c r="A50" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="C50" s="19" t="s">
+      <c r="C50" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="D50" s="19" t="s">
+      <c r="D50" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="3" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="115.2">
-      <c r="A51" s="19" t="s">
+      <c r="A51" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="19" t="s">
+      <c r="B51" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="C51" s="19" t="s">
+      <c r="C51" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="D51" s="19" t="s">
+      <c r="D51" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="3" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="115.2">
-      <c r="A52" s="19" t="s">
+      <c r="A52" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B52" s="19" t="s">
+      <c r="B52" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D52" s="19" t="s">
+      <c r="D52" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="3" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="100.8">
-      <c r="A53" s="19" t="s">
+      <c r="A53" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B53" s="19" t="s">
+      <c r="B53" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="C53" s="19" t="s">
+      <c r="C53" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="D53" s="19" t="s">
+      <c r="D53" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="3" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="100.8">
-      <c r="A54" s="19" t="s">
+      <c r="A54" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B54" s="19" t="s">
+      <c r="B54" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D54" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="3" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="86.4">
-      <c r="A55" s="19" t="s">
+      <c r="A55" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="B55" s="19" t="s">
+      <c r="B55" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="C55" s="19" t="s">
+      <c r="C55" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="D55" s="19" t="s">
+      <c r="D55" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" s="3" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="86.4">
-      <c r="A56" s="19" t="s">
+      <c r="A56" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="B56" s="19" t="s">
+      <c r="B56" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="C56" s="19" t="s">
+      <c r="C56" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="D56" s="19" t="s">
+      <c r="D56" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="E56" s="19" t="s">
+      <c r="E56" s="3" t="s">
         <v>304</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="57.6">
+      <c r="A57" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="57.6">
+      <c r="A58" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="57.6">
+      <c r="A59" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="57.6">
+      <c r="A60" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="43.2">
+      <c r="A61" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="43.2">
+      <c r="A62" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="43.2">
+      <c r="A63" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="57.6">
+      <c r="A64" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>